<commit_message>
feat(planning): add HH mensuales bar chart + monthly summary table
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/Planificación semanal actual .xlsx
+++ b/docs/planning/creador gantt/Planificación semanal actual .xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Planificacion Semanal" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HH Mensuales" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +78,31 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B6B1E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0070AD47"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -140,8 +164,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -163,11 +192,55 @@
         <color rgb="00B4B4B4"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -236,6 +309,41 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -311,6 +419,362 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Horas Hombre por Semana</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>HH por Semana</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="8"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="9"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="F2F2F2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="10"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="11"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="12"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="13"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="14"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="15"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dLbls>
+            <numFmt formatCode="0"/>
+            <showVal val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'HH Mensuales'!$B$5:$Q$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'HH Mensuales'!$B$6:$Q$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Max 15 HH</v>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln w="25000">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'HH Mensuales'!$B$7:$Q$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Semana</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="20"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Horas Hombre (HH)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10800000" cy="5760000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -618,10 +1082,10 @@
           <t>HERMES-A1 — Planificacion Semanal</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="B1" s="29" t="n"/>
+      <c r="C1" s="29" t="n"/>
+      <c r="D1" s="29" t="n"/>
+      <c r="E1" s="30" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -629,10 +1093,10 @@
           <t>Monitoreo Sismico Estructural | FreeRTOS + STM32F446RE | LIND SpA | Junio 2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+      <c r="B2" s="29" t="n"/>
+      <c r="C2" s="29" t="n"/>
+      <c r="D2" s="29" t="n"/>
+      <c r="E2" s="30" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -640,10 +1104,10 @@
           <t>Maximo: 15 HH/semana | Orden cronologico inverso (mas reciente primero) | Sesion actual: [ACTUAL]</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="29" t="n"/>
+      <c r="E3" s="30" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
       <c r="A4" s="6" t="n"/>
@@ -686,10 +1150,10 @@
           <t>Semana 26: 23 al 27 Jun 2026  [SESION ACTUAL]</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="30" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
@@ -805,9 +1269,9 @@
           <t>Total HH: 15 / 15</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="30" t="n"/>
       <c r="E12" s="6" t="n"/>
     </row>
     <row r="13" ht="6" customHeight="1">
@@ -823,10 +1287,10 @@
           <t>Semana 29-30: 14 al 25 Jul 2026</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
+      <c r="B14" s="29" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="30" t="n"/>
     </row>
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -942,9 +1406,9 @@
           <t>Total HH: 15 / 15</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="B19" s="29" t="n"/>
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="30" t="n"/>
       <c r="E19" s="6" t="n"/>
     </row>
     <row r="20" ht="6" customHeight="1">
@@ -960,10 +1424,10 @@
           <t>Semana 28: 07 al 11 Jul 2026</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="30" t="n"/>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
@@ -1079,9 +1543,9 @@
           <t>Total HH: 14 / 15</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="30" t="n"/>
       <c r="E26" s="6" t="n"/>
     </row>
     <row r="27" ht="6" customHeight="1">
@@ -1097,10 +1561,10 @@
           <t>Semana 27: 30 Jun al 04 Jul 2026</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="30" t="n"/>
     </row>
     <row r="29" ht="52" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -1216,9 +1680,9 @@
           <t>Total HH: 14 / 15</t>
         </is>
       </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="30" t="n"/>
       <c r="E33" s="6" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1">
@@ -1234,10 +1698,10 @@
           <t>Semana 24: 09 al 13 Jun 2026</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
+      <c r="B35" s="29" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="30" t="n"/>
     </row>
     <row r="36" ht="52" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
@@ -1353,9 +1817,9 @@
           <t>Total HH: 15 / 15</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
+      <c r="B40" s="29" t="n"/>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="30" t="n"/>
       <c r="E40" s="6" t="n"/>
     </row>
     <row r="41" ht="6" customHeight="1">
@@ -1371,10 +1835,10 @@
           <t>Semana 23: 02 al 06 Jun 2026</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
+      <c r="B42" s="29" t="n"/>
+      <c r="C42" s="29" t="n"/>
+      <c r="D42" s="29" t="n"/>
+      <c r="E42" s="30" t="n"/>
     </row>
     <row r="43" ht="52" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
@@ -1490,9 +1954,9 @@
           <t>Total HH: 15 / 15</t>
         </is>
       </c>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="29" t="n"/>
+      <c r="D47" s="30" t="n"/>
       <c r="E47" s="6" t="n"/>
     </row>
     <row r="48" ht="6" customHeight="1">
@@ -1508,10 +1972,10 @@
           <t>Semana 22: 25 al 29 May</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
+      <c r="B49" s="29" t="n"/>
+      <c r="C49" s="29" t="n"/>
+      <c r="D49" s="29" t="n"/>
+      <c r="E49" s="30" t="n"/>
     </row>
     <row r="50" ht="52" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
@@ -1627,9 +2091,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="6" t="n"/>
-      <c r="D54" s="6" t="n"/>
+      <c r="B54" s="29" t="n"/>
+      <c r="C54" s="29" t="n"/>
+      <c r="D54" s="30" t="n"/>
       <c r="E54" s="6" t="n"/>
     </row>
     <row r="55" ht="6" customHeight="1">
@@ -1645,10 +2109,10 @@
           <t>Semana 21: 18 al 22 May</t>
         </is>
       </c>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
+      <c r="B56" s="29" t="n"/>
+      <c r="C56" s="29" t="n"/>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="30" t="n"/>
     </row>
     <row r="57" ht="52" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
@@ -1764,9 +2228,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
+      <c r="B61" s="29" t="n"/>
+      <c r="C61" s="29" t="n"/>
+      <c r="D61" s="30" t="n"/>
       <c r="E61" s="6" t="n"/>
     </row>
     <row r="62" ht="6" customHeight="1">
@@ -1782,10 +2246,10 @@
           <t>Semana 20: 11 al 15 May</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="n"/>
+      <c r="B63" s="29" t="n"/>
+      <c r="C63" s="29" t="n"/>
+      <c r="D63" s="29" t="n"/>
+      <c r="E63" s="30" t="n"/>
     </row>
     <row r="64" ht="52" customHeight="1">
       <c r="A64" s="10" t="inlineStr">
@@ -1901,9 +2365,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="6" t="n"/>
-      <c r="D68" s="6" t="n"/>
+      <c r="B68" s="29" t="n"/>
+      <c r="C68" s="29" t="n"/>
+      <c r="D68" s="30" t="n"/>
       <c r="E68" s="6" t="n"/>
     </row>
     <row r="69" ht="6" customHeight="1">
@@ -1919,10 +2383,10 @@
           <t>Semana 19: 04 al 08 May</t>
         </is>
       </c>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
+      <c r="B70" s="29" t="n"/>
+      <c r="C70" s="29" t="n"/>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="30" t="n"/>
     </row>
     <row r="71" ht="52" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
@@ -2038,9 +2502,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B75" s="6" t="n"/>
-      <c r="C75" s="6" t="n"/>
-      <c r="D75" s="6" t="n"/>
+      <c r="B75" s="29" t="n"/>
+      <c r="C75" s="29" t="n"/>
+      <c r="D75" s="30" t="n"/>
       <c r="E75" s="6" t="n"/>
     </row>
     <row r="76" ht="6" customHeight="1">
@@ -2056,10 +2520,10 @@
           <t>Semana 18: 27 Abr al 01 May</t>
         </is>
       </c>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="2" t="n"/>
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="29" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="30" t="n"/>
     </row>
     <row r="78" ht="52" customHeight="1">
       <c r="A78" s="10" t="inlineStr">
@@ -2175,9 +2639,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B82" s="6" t="n"/>
-      <c r="C82" s="6" t="n"/>
-      <c r="D82" s="6" t="n"/>
+      <c r="B82" s="29" t="n"/>
+      <c r="C82" s="29" t="n"/>
+      <c r="D82" s="30" t="n"/>
       <c r="E82" s="6" t="n"/>
     </row>
     <row r="83" ht="6" customHeight="1">
@@ -2193,10 +2657,10 @@
           <t>Semana 17: 20 al 24 Abril</t>
         </is>
       </c>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
-      <c r="E84" s="2" t="n"/>
+      <c r="B84" s="29" t="n"/>
+      <c r="C84" s="29" t="n"/>
+      <c r="D84" s="29" t="n"/>
+      <c r="E84" s="30" t="n"/>
     </row>
     <row r="85" ht="52" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
@@ -2312,9 +2776,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="6" t="n"/>
+      <c r="B89" s="29" t="n"/>
+      <c r="C89" s="29" t="n"/>
+      <c r="D89" s="30" t="n"/>
       <c r="E89" s="6" t="n"/>
     </row>
     <row r="90" ht="6" customHeight="1">
@@ -2330,10 +2794,10 @@
           <t>Semana 16: 13 al 17 Abril</t>
         </is>
       </c>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
+      <c r="B91" s="29" t="n"/>
+      <c r="C91" s="29" t="n"/>
+      <c r="D91" s="29" t="n"/>
+      <c r="E91" s="30" t="n"/>
     </row>
     <row r="92" ht="52" customHeight="1">
       <c r="A92" s="10" t="inlineStr">
@@ -2449,9 +2913,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B96" s="6" t="n"/>
-      <c r="C96" s="6" t="n"/>
-      <c r="D96" s="6" t="n"/>
+      <c r="B96" s="29" t="n"/>
+      <c r="C96" s="29" t="n"/>
+      <c r="D96" s="30" t="n"/>
       <c r="E96" s="6" t="n"/>
     </row>
     <row r="97" ht="6" customHeight="1">
@@ -2467,10 +2931,10 @@
           <t>Semana 15: 06 al 10 Abril</t>
         </is>
       </c>
-      <c r="B98" s="2" t="n"/>
-      <c r="C98" s="2" t="n"/>
-      <c r="D98" s="2" t="n"/>
-      <c r="E98" s="2" t="n"/>
+      <c r="B98" s="29" t="n"/>
+      <c r="C98" s="29" t="n"/>
+      <c r="D98" s="29" t="n"/>
+      <c r="E98" s="30" t="n"/>
     </row>
     <row r="99" ht="52" customHeight="1">
       <c r="A99" s="10" t="inlineStr">
@@ -2586,9 +3050,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B103" s="6" t="n"/>
-      <c r="C103" s="6" t="n"/>
-      <c r="D103" s="6" t="n"/>
+      <c r="B103" s="29" t="n"/>
+      <c r="C103" s="29" t="n"/>
+      <c r="D103" s="30" t="n"/>
       <c r="E103" s="6" t="n"/>
     </row>
     <row r="104" ht="6" customHeight="1">
@@ -2604,10 +3068,10 @@
           <t>Semana 14: 01 al 02 Abril</t>
         </is>
       </c>
-      <c r="B105" s="2" t="n"/>
-      <c r="C105" s="2" t="n"/>
-      <c r="D105" s="2" t="n"/>
-      <c r="E105" s="2" t="n"/>
+      <c r="B105" s="29" t="n"/>
+      <c r="C105" s="29" t="n"/>
+      <c r="D105" s="29" t="n"/>
+      <c r="E105" s="30" t="n"/>
     </row>
     <row r="106" ht="52" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
@@ -2723,9 +3187,9 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B110" s="6" t="n"/>
-      <c r="C110" s="6" t="n"/>
-      <c r="D110" s="6" t="n"/>
+      <c r="B110" s="29" t="n"/>
+      <c r="C110" s="29" t="n"/>
+      <c r="D110" s="30" t="n"/>
       <c r="E110" s="6" t="n"/>
     </row>
     <row r="111" ht="6" customHeight="1">
@@ -2741,10 +3205,10 @@
           <t>📌 Planificación generada desde GANTT 2026 — Semana actual: 25 (16-20 Jun 2026)</t>
         </is>
       </c>
-      <c r="B112" s="2" t="n"/>
-      <c r="C112" s="2" t="n"/>
-      <c r="D112" s="2" t="n"/>
-      <c r="E112" s="2" t="n"/>
+      <c r="B112" s="29" t="n"/>
+      <c r="C112" s="29" t="n"/>
+      <c r="D112" s="29" t="n"/>
+      <c r="E112" s="30" t="n"/>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="16" t="inlineStr">
@@ -2752,21 +3216,22 @@
           <t>Total HH: 0 / 15</t>
         </is>
       </c>
-      <c r="B113" s="6" t="n"/>
-      <c r="C113" s="6" t="n"/>
-      <c r="D113" s="6" t="n"/>
+      <c r="B113" s="29" t="n"/>
+      <c r="C113" s="29" t="n"/>
+      <c r="D113" s="30" t="n"/>
       <c r="E113" s="6" t="n"/>
     </row>
+    <row r="114"/>
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="18" t="inlineStr">
         <is>
           <t>TAREAS EN PROGRESO</t>
         </is>
       </c>
-      <c r="B115" s="19" t="n"/>
-      <c r="C115" s="19" t="n"/>
-      <c r="D115" s="19" t="n"/>
-      <c r="E115" s="19" t="n"/>
+      <c r="B115" s="29" t="n"/>
+      <c r="C115" s="29" t="n"/>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="30" t="n"/>
     </row>
     <row r="116" ht="32" customHeight="1">
       <c r="A116" s="20" t="inlineStr">
@@ -2779,9 +3244,9 @@
           <t>Migración de interrupción Wake-on-Motion a NVIC con CMSIS-RTOS v2. Requiere refactorización del manejo de interrupciones del ADXL355 desde el modelo bare-metal al modelo RTOS con event flags. La rutina de interrupción debe señalizar a sensor_task en lugar de manejar datos directamente. [3 HH]</t>
         </is>
       </c>
-      <c r="C116" s="22" t="n"/>
-      <c r="D116" s="22" t="n"/>
-      <c r="E116" s="22" t="n"/>
+      <c r="C116" s="29" t="n"/>
+      <c r="D116" s="29" t="n"/>
+      <c r="E116" s="30" t="n"/>
     </row>
     <row r="117" ht="32" customHeight="1">
       <c r="A117" s="20" t="inlineStr">
@@ -2794,9 +3259,9 @@
           <t>Pruebas de compilación cruzada y validación de enlace. Verificar que todas las dependencias entre módulos estén correctamente vinculadas en el nuevo proyecto CMSIS. Resolver posibles errores L6218E (símbolos no resueltos) en la toolchain ARM GCC. [2 HH]</t>
         </is>
       </c>
-      <c r="C117" s="22" t="n"/>
-      <c r="D117" s="22" t="n"/>
-      <c r="E117" s="22" t="n"/>
+      <c r="C117" s="29" t="n"/>
+      <c r="D117" s="29" t="n"/>
+      <c r="E117" s="30" t="n"/>
     </row>
     <row r="118" ht="32" customHeight="1">
       <c r="A118" s="20" t="inlineStr">
@@ -2809,20 +3274,21 @@
           <t>Implementación de script de automatización de flasheo y prueba. Crear script para automatizar flasheo vía OpenOCD y captura de logs seriales para pruebas repetibles. [2 HH]</t>
         </is>
       </c>
-      <c r="C118" s="22" t="n"/>
-      <c r="D118" s="22" t="n"/>
-      <c r="E118" s="22" t="n"/>
-    </row>
+      <c r="C118" s="29" t="n"/>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="30" t="n"/>
+    </row>
+    <row r="119"/>
     <row r="120" ht="28" customHeight="1">
       <c r="A120" s="23" t="inlineStr">
         <is>
           <t>TAREAS FUTURAS</t>
         </is>
       </c>
-      <c r="B120" s="24" t="n"/>
-      <c r="C120" s="24" t="n"/>
-      <c r="D120" s="24" t="n"/>
-      <c r="E120" s="24" t="n"/>
+      <c r="B120" s="29" t="n"/>
+      <c r="C120" s="29" t="n"/>
+      <c r="D120" s="29" t="n"/>
+      <c r="E120" s="30" t="n"/>
     </row>
     <row r="121" ht="32" customHeight="1">
       <c r="A121" s="25" t="inlineStr">
@@ -2835,9 +3301,9 @@
           <t>Port de ADXL355 a ADXL312. Evaluar compatibilidad de pines y registros del ADXL312 (acelerómetro de bajo costo) como reemplazo del ADXL355. Adaptar driver SPI y lógica de configuración. Estimación: 6 HH.</t>
         </is>
       </c>
-      <c r="C121" s="27" t="n"/>
-      <c r="D121" s="27" t="n"/>
-      <c r="E121" s="27" t="n"/>
+      <c r="C121" s="29" t="n"/>
+      <c r="D121" s="29" t="n"/>
+      <c r="E121" s="30" t="n"/>
     </row>
     <row r="122" ht="32" customHeight="1">
       <c r="A122" s="25" t="inlineStr">
@@ -2850,9 +3316,9 @@
           <t>Implementación de pruebas unitarias para módulos RTOS. Desarrollar pruebas para sensor_task, file_task, modem_task usando un framework de pruebas embebido (CMock/Unity). Validar transiciones de estado y manejo de errores. Estimación: 8 HH.</t>
         </is>
       </c>
-      <c r="C122" s="27" t="n"/>
-      <c r="D122" s="27" t="n"/>
-      <c r="E122" s="27" t="n"/>
+      <c r="C122" s="29" t="n"/>
+      <c r="D122" s="29" t="n"/>
+      <c r="E122" s="30" t="n"/>
     </row>
     <row r="123" ht="32" customHeight="1">
       <c r="A123" s="25" t="inlineStr">
@@ -2865,9 +3331,9 @@
           <t>Integración con backend IoT. Desarrollar firmware de comunicación MQTT sobre PPP/EC25 para publicación periódica de datos de vibración. Implementar mecanismo de buffer local con reenvío en caso de fallo de conectividad. Estimación: 10 HH.</t>
         </is>
       </c>
-      <c r="C123" s="27" t="n"/>
-      <c r="D123" s="27" t="n"/>
-      <c r="E123" s="27" t="n"/>
+      <c r="C123" s="29" t="n"/>
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="30" t="n"/>
     </row>
     <row r="124" ht="32" customHeight="1">
       <c r="A124" s="25" t="inlineStr">
@@ -2880,9 +3346,9 @@
           <t>Reducción de consumo energético. Implementar modos de bajo consumo (STOP/SLEEP) del STM32F446RE entre ciclos de adquisición. Configurar wake-up por RTC o interrupción de sensor. Estimación: 8 HH.</t>
         </is>
       </c>
-      <c r="C124" s="27" t="n"/>
-      <c r="D124" s="27" t="n"/>
-      <c r="E124" s="27" t="n"/>
+      <c r="C124" s="29" t="n"/>
+      <c r="D124" s="29" t="n"/>
+      <c r="E124" s="30" t="n"/>
     </row>
     <row r="125" ht="32" customHeight="1">
       <c r="A125" s="25" t="inlineStr">
@@ -2895,10 +3361,12 @@
           <t>Diseño de PCB definitivo. Diseñar esquemático y layout de PCB para el sistema de monitoreo de vibraciones con STM32F446RE, ADXL355/ADXL312, Quectel EC25 y alimentación por batería. Estimación: 20 HH.</t>
         </is>
       </c>
-      <c r="C125" s="27" t="n"/>
-      <c r="D125" s="27" t="n"/>
-      <c r="E125" s="27" t="n"/>
-    </row>
+      <c r="C125" s="29" t="n"/>
+      <c r="D125" s="29" t="n"/>
+      <c r="E125" s="30" t="n"/>
+    </row>
+    <row r="126"/>
+    <row r="127"/>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="28" t="inlineStr">
         <is>
@@ -2917,8 +3385,8 @@
     <mergeCell ref="B124:E124"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A70:E70"/>
+    <mergeCell ref="B123:E123"/>
     <mergeCell ref="A68:D68"/>
-    <mergeCell ref="B123:E123"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A128:E128"/>
@@ -2958,4 +3426,485 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>HERMES-A1 — Horas Hombre Mensuales por Semana</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Grafico de barras agrupado por mes | Maximo: 15 HH/semana | LIND SpA | Junio 2026</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Jan 2025</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="33" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="33" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">📌 Planificación generada </t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 14:
+(01-02 Abril)</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 15:
+(06-10 Abril)</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 16:
+(13-17 Abril)</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 17:
+(20-24 Abril)</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>Semana 18: 27 Abr al 01 M</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 19:
+(04-08 May)</t>
+        </is>
+      </c>
+      <c r="I5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 20:
+(11-15 May)</t>
+        </is>
+      </c>
+      <c r="J5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 21:
+(18-22 May)</t>
+        </is>
+      </c>
+      <c r="K5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 22:
+(25-29 May)</t>
+        </is>
+      </c>
+      <c r="L5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 23:
+(02-06 Jun)</t>
+        </is>
+      </c>
+      <c r="M5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 24:
+(09-13 Jun)</t>
+        </is>
+      </c>
+      <c r="N5" s="35" t="inlineStr">
+        <is>
+          <t>Sem 26:
+(23-27 Jun)</t>
+        </is>
+      </c>
+      <c r="O5" s="34" t="inlineStr">
+        <is>
+          <t>Semana 27: 30 Jun al 04 J</t>
+        </is>
+      </c>
+      <c r="P5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 28:
+(07-11 Jul)</t>
+        </is>
+      </c>
+      <c r="Q5" s="34" t="inlineStr">
+        <is>
+          <t>Sem 29-30:
+(14-25 Jul)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="37" t="n">
+        <v>14</v>
+      </c>
+      <c r="P6" s="37" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q6" s="37" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="G7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="J7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="K7" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="L7" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="M7" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="N7" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="O7" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="P7" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q7" s="37" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="39" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="D8" s="40" t="n"/>
+      <c r="E8" s="40" t="n"/>
+      <c r="F8" s="40" t="n"/>
+      <c r="G8" s="40" t="n"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="I8" s="40" t="n"/>
+      <c r="J8" s="40" t="n"/>
+      <c r="K8" s="40" t="n"/>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>59 HH total</t>
+        </is>
+      </c>
+      <c r="M8" s="40" t="n"/>
+      <c r="N8" s="40" t="n"/>
+      <c r="O8" s="40" t="n"/>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>29 HH total</t>
+        </is>
+      </c>
+      <c r="Q8" s="40" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>Generado automaticamente | Actualizado: 24 Junio 2026 | LIND SpA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Resumen por Mes</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Semanas</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>HH Total</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>HH Promedio</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>January 2025</t>
+        </is>
+      </c>
+      <c r="B35" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="B36" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B37" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" s="42" t="n">
+        <v>59</v>
+      </c>
+      <c r="D38" s="43" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="B39" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="42" t="n">
+        <v>29</v>
+      </c>
+      <c r="D39" s="43" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="C8:G8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: .DONE marker timing + start.ps1 auto-tunnel + dossier v2.0
- modem_task.c: HAL_Delay(50) after f_close for SD NAND program completion
- start.ps1: full auto-start (Flask + cloudflared + credentials.h update)
- credentials.h: updated tunnel URL
- docs: dossier v2.0 HTML + PDF generation scripts
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/Planificación semanal actual .xlsx
+++ b/docs/planning/creador gantt/Planificación semanal actual .xlsx
@@ -448,7 +448,7 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>HH por Semana</v>
+            <v>HH Semanal</v>
           </tx>
           <spPr>
             <a:ln>
@@ -659,9 +659,6 @@
             <v>Max 15 HH</v>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="C00000"/>
-            </a:solidFill>
             <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="C00000"/>
@@ -677,9 +674,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <showVal val="0"/>
+          </dLbls>
           <val>
             <numRef>
-              <f>'HH Mensuales'!$B$7:$Q$7</f>
+              <f>'HH Mensuales'!$B$10:$Q$10</f>
             </numRef>
           </val>
         </ser>
@@ -701,7 +701,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Semana</a:t>
+                  <a:t/>
                 </a:r>
               </a:p>
             </rich>
@@ -720,7 +720,6 @@
           <min val="0"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -742,7 +741,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -756,10 +755,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10800000" cy="5760000"/>
+    <ext cx="11520000" cy="6480000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -3434,7 +3433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3470,7 +3469,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="32" t="inlineStr">
         <is>
-          <t>Grafico de barras agrupado por mes | Maximo: 15 HH/semana | LIND SpA | Junio 2026</t>
+          <t>Grafico de barras | Maximo: 15 HH/semana | LIND SpA | Junio 2026</t>
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
@@ -3478,6 +3477,7 @@
       <c r="D2" s="5" t="n"/>
       <c r="E2" s="5" t="n"/>
     </row>
+    <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="33" t="inlineStr">
         <is>
@@ -3662,247 +3662,328 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="38" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="n">
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="G7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="H7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="I7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="J7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="K7" s="36" t="inlineStr">
+        <is>
+          <t>Sin HH</t>
+        </is>
+      </c>
+      <c r="L7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="N7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="O7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="P7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q7" s="37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="6" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="39" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="n"/>
+      <c r="E9" s="40" t="n"/>
+      <c r="F9" s="40" t="n"/>
+      <c r="G9" s="40" t="n"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>0 HH total</t>
+        </is>
+      </c>
+      <c r="I9" s="40" t="n"/>
+      <c r="J9" s="40" t="n"/>
+      <c r="K9" s="40" t="n"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>59 HH total</t>
+        </is>
+      </c>
+      <c r="M9" s="40" t="n"/>
+      <c r="N9" s="40" t="n"/>
+      <c r="O9" s="40" t="n"/>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>29 HH total</t>
+        </is>
+      </c>
+      <c r="Q9" s="40" t="n"/>
+    </row>
+    <row r="10" ht="4" customHeight="1">
+      <c r="A10" s="39" t="inlineStr"/>
+      <c r="B10" t="n">
         <v>15</v>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C10" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D10" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="36" t="n">
+      <c r="E10" t="n">
         <v>15</v>
       </c>
-      <c r="F7" s="36" t="n">
+      <c r="F10" t="n">
         <v>15</v>
       </c>
-      <c r="G7" s="36" t="n">
+      <c r="G10" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="36" t="n">
+      <c r="H10" t="n">
         <v>15</v>
       </c>
-      <c r="I7" s="36" t="n">
+      <c r="I10" t="n">
         <v>15</v>
       </c>
-      <c r="J7" s="36" t="n">
+      <c r="J10" t="n">
         <v>15</v>
       </c>
-      <c r="K7" s="36" t="n">
+      <c r="K10" t="n">
         <v>15</v>
       </c>
-      <c r="L7" s="37" t="n">
+      <c r="L10" t="n">
         <v>15</v>
       </c>
-      <c r="M7" s="37" t="n">
+      <c r="M10" t="n">
         <v>15</v>
       </c>
-      <c r="N7" s="37" t="n">
+      <c r="N10" t="n">
         <v>15</v>
       </c>
-      <c r="O7" s="37" t="n">
+      <c r="O10" t="n">
         <v>15</v>
       </c>
-      <c r="P7" s="37" t="n">
+      <c r="P10" t="n">
         <v>15</v>
       </c>
-      <c r="Q7" s="37" t="n">
+      <c r="Q10" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="39" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>0 HH total</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>0 HH total</t>
-        </is>
-      </c>
-      <c r="D8" s="40" t="n"/>
-      <c r="E8" s="40" t="n"/>
-      <c r="F8" s="40" t="n"/>
-      <c r="G8" s="40" t="n"/>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>0 HH total</t>
-        </is>
-      </c>
-      <c r="I8" s="40" t="n"/>
-      <c r="J8" s="40" t="n"/>
-      <c r="K8" s="40" t="n"/>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>59 HH total</t>
-        </is>
-      </c>
-      <c r="M8" s="40" t="n"/>
-      <c r="N8" s="40" t="n"/>
-      <c r="O8" s="40" t="n"/>
-      <c r="P8" s="7" t="inlineStr">
-        <is>
-          <t>29 HH total</t>
-        </is>
-      </c>
-      <c r="Q8" s="40" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Resumen por Mes</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Semanas</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>HH Total</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>HH Promedio</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>January 2025</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="42" t="n">
+        <v>59</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="42" t="n">
+        <v>29</v>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
         <is>
           <t>Generado automaticamente | Actualizado: 24 Junio 2026 | LIND SpA</t>
         </is>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="17" t="inlineStr">
-        <is>
-          <t>Resumen por Mes</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Semanas</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>HH Total</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>HH Promedio</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="41" t="inlineStr">
-        <is>
-          <t>January 2025</t>
-        </is>
-      </c>
-      <c r="B35" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="41" t="inlineStr">
-        <is>
-          <t>April 2026</t>
-        </is>
-      </c>
-      <c r="B36" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="C36" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="41" t="inlineStr">
-        <is>
-          <t>May 2026</t>
-        </is>
-      </c>
-      <c r="B37" s="36" t="n">
-        <v>4</v>
-      </c>
-      <c r="C37" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="43" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="41" t="inlineStr">
-        <is>
-          <t>June 2026</t>
-        </is>
-      </c>
-      <c r="B38" s="36" t="n">
-        <v>4</v>
-      </c>
-      <c r="C38" s="42" t="n">
-        <v>59</v>
-      </c>
-      <c r="D38" s="43" t="n">
-        <v>14.8</v>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="41" t="inlineStr">
-        <is>
-          <t>July 2026</t>
-        </is>
-      </c>
-      <c r="B39" s="36" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" s="42" t="n">
-        <v>29</v>
-      </c>
-      <c r="D39" s="43" t="n">
-        <v>14.5</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="C40" s="7" t="n">
-        <v>88</v>
-      </c>
-      <c r="D40" s="7" t="n">
-        <v>5.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="P9:Q9"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="H9:K9"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="L9:O9"/>
     <mergeCell ref="L4:O4"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>